<commit_message>
Solicitud Humanos y Glosario Finanzas
</commit_message>
<xml_diff>
--- a/wwwroot/templates/siisu.xlsx
+++ b/wwwroot/templates/siisu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UV\Desktop\UV\Solicitud-UV\SSP\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BBAB973-25A5-4332-B54B-E7FEDA14FD12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBAFC6B6-3A42-4BF6-9ECC-DF49F40C1E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -693,8 +693,122 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="justify" wrapText="1"/>
@@ -719,120 +833,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1187,36 +1187,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="25"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="31"/>
     </row>
     <row r="2" spans="1:21" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="28"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="34"/>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
@@ -1228,58 +1228,58 @@
       <c r="U2" s="3"/>
     </row>
     <row r="3" spans="1:21" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="31"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="37"/>
     </row>
     <row r="4" spans="1:21" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:21" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="38" t="s">
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="39"/>
+      <c r="I5" s="39"/>
+      <c r="J5" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="39"/>
-      <c r="L5" s="40"/>
+      <c r="K5" s="45"/>
+      <c r="L5" s="46"/>
     </row>
     <row r="6" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="C6" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
-      <c r="I6" s="35"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
       <c r="J6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1291,15 +1291,15 @@
       </c>
     </row>
     <row r="7" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="42"/>
-      <c r="B7" s="44"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
+      <c r="A7" s="48"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="52"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
       <c r="J7" s="9" t="s">
         <v>34</v>
       </c>
@@ -1314,34 +1314,34 @@
       <c r="A8" s="1"/>
     </row>
     <row r="9" spans="1:21" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="47" t="s">
+      <c r="A9" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="48"/>
-      <c r="C9" s="48"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="47" t="s">
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="48"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="48" t="s">
+      <c r="H9" s="15"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="K9" s="48"/>
-      <c r="L9" s="49"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="16"/>
     </row>
     <row r="10" spans="1:21" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="54" t="s">
+      <c r="B10" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="55"/>
-      <c r="D10" s="56"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="24"/>
       <c r="E10" s="7" t="s">
         <v>7</v>
       </c>
@@ -1360,20 +1360,20 @@
       <c r="J10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K10" s="51" t="s">
+      <c r="K10" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="L10" s="52"/>
+      <c r="L10" s="20"/>
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="57" t="s">
+      <c r="B11" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="58"/>
-      <c r="D11" s="59"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="27"/>
       <c r="E11" s="12" t="s">
         <v>28</v>
       </c>
@@ -1392,138 +1392,153 @@
       <c r="J11" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="K11" s="53"/>
-      <c r="L11" s="53"/>
-    </row>
-    <row r="12" spans="1:21" s="6" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K11" s="21"/>
+      <c r="L11" s="21"/>
+    </row>
+    <row r="12" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="18"/>
     </row>
     <row r="13" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="14"/>
-    </row>
-    <row r="14" spans="1:21" s="6" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K13" s="18"/>
+      <c r="L13" s="18"/>
+    </row>
+    <row r="14" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
-      <c r="B14" s="50"/>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="18"/>
     </row>
     <row r="15" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
       <c r="I15" s="13"/>
       <c r="J15" s="13"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
     </row>
     <row r="16" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="18"/>
     </row>
     <row r="17" spans="1:12" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" spans="1:12" ht="114" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="54"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="54"/>
+      <c r="J18" s="54"/>
+      <c r="K18" s="54"/>
+      <c r="L18" s="54"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="18"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
+      <c r="A19" s="56"/>
+      <c r="B19" s="56"/>
+      <c r="C19" s="56"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="56"/>
+      <c r="F19" s="56"/>
+      <c r="G19" s="56"/>
+      <c r="H19" s="56"/>
+      <c r="I19" s="56"/>
+      <c r="J19" s="56"/>
+      <c r="K19" s="56"/>
+      <c r="L19" s="56"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
+      <c r="B20" s="57"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="57"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="57"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="55"/>
+      <c r="F21" s="55"/>
+      <c r="G21" s="55"/>
       <c r="I21" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J21" s="20" t="s">
+      <c r="J21" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="K21" s="21"/>
-      <c r="L21" s="22"/>
+      <c r="K21" s="59"/>
+      <c r="L21" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="D6:I7"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
@@ -1540,21 +1555,6 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="G9:I9"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="D6:I7"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="A18:L18"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="J21:L21"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
Solicitudes Tabla CRUD y Login
</commit_message>
<xml_diff>
--- a/wwwroot/templates/siisu.xlsx
+++ b/wwwroot/templates/siisu.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UV\Desktop\UV\Solicitud-UV\SSP\wwwroot\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UV\Desktop\UV\Solicitud-UV\Github\SSP\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBAFC6B6-3A42-4BF6-9ECC-DF49F40C1E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB57E8C-A81F-48C4-8168-E6C5B8D15CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -306,7 +306,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -430,43 +430,6 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -652,7 +615,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -672,19 +635,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -717,24 +680,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -744,7 +689,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -753,7 +698,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -771,15 +716,15 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -792,47 +737,53 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="justify" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="justify"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1187,36 +1138,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="31"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="25"/>
     </row>
     <row r="2" spans="1:21" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="34"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="28"/>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
@@ -1228,58 +1179,58 @@
       <c r="U2" s="3"/>
     </row>
     <row r="3" spans="1:21" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="37"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="31"/>
     </row>
     <row r="4" spans="1:21" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:21" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="39"/>
-      <c r="J5" s="44" t="s">
+      <c r="B5" s="33"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="45"/>
-      <c r="L5" s="46"/>
+      <c r="K5" s="39"/>
+      <c r="L5" s="40"/>
     </row>
     <row r="6" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="49" t="s">
+      <c r="B6" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="51" t="s">
+      <c r="C6" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="35"/>
       <c r="J6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1291,15 +1242,15 @@
       </c>
     </row>
     <row r="7" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="48"/>
-      <c r="B7" s="50"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="42"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="43"/>
-      <c r="I7" s="43"/>
+      <c r="A7" s="42"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
       <c r="J7" s="9" t="s">
         <v>34</v>
       </c>
@@ -1337,11 +1288,11 @@
       <c r="A10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="24"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="7" t="s">
         <v>7</v>
       </c>
@@ -1369,11 +1320,11 @@
       <c r="A11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="26"/>
-      <c r="D11" s="27"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="55"/>
       <c r="E11" s="12" t="s">
         <v>28</v>
       </c>
@@ -1397,9 +1348,9 @@
     </row>
     <row r="12" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
@@ -1467,60 +1418,60 @@
     </row>
     <row r="17" spans="1:12" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" spans="1:12" ht="114" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="53" t="s">
+      <c r="A18" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="54"/>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="54"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="54"/>
-      <c r="I18" s="54"/>
-      <c r="J18" s="54"/>
-      <c r="K18" s="54"/>
-      <c r="L18" s="54"/>
+      <c r="B18" s="48"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="48"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="48"/>
+      <c r="K18" s="48"/>
+      <c r="L18" s="48"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="56"/>
-      <c r="B19" s="56"/>
-      <c r="C19" s="56"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="56"/>
-      <c r="J19" s="56"/>
-      <c r="K19" s="56"/>
-      <c r="L19" s="56"/>
+      <c r="A19" s="50"/>
+      <c r="B19" s="50"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+      <c r="L19" s="50"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="57"/>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
+      <c r="B20" s="51"/>
+      <c r="C20" s="51"/>
+      <c r="D20" s="51"/>
+      <c r="E20" s="51"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="51"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="55" t="s">
+      <c r="B21" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="55"/>
-      <c r="D21" s="55"/>
-      <c r="E21" s="55"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="55"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
+      <c r="G21" s="49"/>
       <c r="I21" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J21" s="58" t="s">
+      <c r="J21" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="K21" s="59"/>
-      <c r="L21" s="60"/>
+      <c r="K21" s="53"/>
+      <c r="L21" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="31">

</xml_diff>

<commit_message>
Optimizar Tabs Solicitud y Permisos, pendiente Humanos
</commit_message>
<xml_diff>
--- a/wwwroot/templates/siisu.xlsx
+++ b/wwwroot/templates/siisu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UV\Desktop\UV\Solicitud-UV\Github\SSP\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB57E8C-A81F-48C4-8168-E6C5B8D15CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F5BFD4-2AB1-48B5-AD41-4F14D5BAB6C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="15600" tabRatio="602" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formato" sheetId="1" r:id="rId1"/>
@@ -656,6 +656,105 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -668,9 +767,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -679,111 +775,15 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1126,12 +1126,13 @@
   <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="10" customWidth="1"/>
     <col min="4" max="4" width="7.7109375" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" customWidth="1"/>
     <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.42578125" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="12.5703125" customWidth="1"/>
     <col min="12" max="12" width="9.85546875" customWidth="1"/>
@@ -1265,34 +1266,34 @@
       <c r="A8" s="1"/>
     </row>
     <row r="9" spans="1:21" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="14" t="s">
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="15"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="15" t="s">
+      <c r="H9" s="48"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="K9" s="15"/>
-      <c r="L9" s="16"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="49"/>
     </row>
     <row r="10" spans="1:21" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="56"/>
-      <c r="D10" s="20"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="52"/>
       <c r="E10" s="7" t="s">
         <v>7</v>
       </c>
@@ -1311,10 +1312,10 @@
       <c r="J10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K10" s="19" t="s">
+      <c r="K10" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="L10" s="20"/>
+      <c r="L10" s="52"/>
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
@@ -1343,153 +1344,138 @@
       <c r="J11" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="K11" s="21"/>
-      <c r="L11" s="21"/>
+      <c r="K11" s="53"/>
+      <c r="L11" s="53"/>
     </row>
     <row r="12" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
+      <c r="B12" s="56"/>
+      <c r="C12" s="56"/>
+      <c r="D12" s="56"/>
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="14"/>
     </row>
     <row r="13" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="18"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="14"/>
     </row>
     <row r="14" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
+      <c r="B14" s="50"/>
+      <c r="C14" s="50"/>
+      <c r="D14" s="50"/>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
+      <c r="K14" s="14"/>
+      <c r="L14" s="14"/>
     </row>
     <row r="15" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
       <c r="I15" s="13"/>
       <c r="J15" s="13"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
+      <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
     </row>
     <row r="16" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
     </row>
     <row r="17" spans="1:12" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" spans="1:12" ht="114" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="47" t="s">
+      <c r="A18" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="48"/>
-      <c r="C18" s="48"/>
-      <c r="D18" s="48"/>
-      <c r="E18" s="48"/>
-      <c r="F18" s="48"/>
-      <c r="G18" s="48"/>
-      <c r="H18" s="48"/>
-      <c r="I18" s="48"/>
-      <c r="J18" s="48"/>
-      <c r="K18" s="48"/>
-      <c r="L18" s="48"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="50"/>
-      <c r="B19" s="50"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="50"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
-      <c r="L19" s="50"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="18"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="51"/>
-      <c r="C20" s="51"/>
-      <c r="D20" s="51"/>
-      <c r="E20" s="51"/>
-      <c r="F20" s="51"/>
-      <c r="G20" s="51"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="49" t="s">
+      <c r="B21" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="49"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="49"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
       <c r="I21" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J21" s="52" t="s">
+      <c r="J21" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="K21" s="53"/>
-      <c r="L21" s="54"/>
+      <c r="K21" s="21"/>
+      <c r="L21" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="A18:L18"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="D6:I7"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
@@ -1506,6 +1492,21 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="G9:I9"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="D6:I7"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="J21:L21"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
Actualizar Solicitud, Dependencia en Documentos y Usuario RH Adicional
</commit_message>
<xml_diff>
--- a/wwwroot/templates/siisu.xlsx
+++ b/wwwroot/templates/siisu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UV\Desktop\UV\Solicitud-UV\Github\SSP\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F5BFD4-2AB1-48B5-AD41-4F14D5BAB6C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5496824-1A8E-4461-8FD7-B8C60F6B8CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="15600" tabRatio="602" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -656,8 +656,98 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="justify" wrapText="1"/>
@@ -683,107 +773,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1126,8 +1126,9 @@
   <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" customWidth="1"/>
+    <col min="3" max="4" width="10.85546875" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" customWidth="1"/>
     <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -1139,36 +1140,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="27"/>
     </row>
     <row r="2" spans="1:21" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="28"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="30"/>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
@@ -1180,58 +1181,58 @@
       <c r="U2" s="3"/>
     </row>
     <row r="3" spans="1:21" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="31"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:21" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:21" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="38" t="s">
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="39"/>
-      <c r="L5" s="40"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="38"/>
     </row>
     <row r="6" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="C6" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
-      <c r="I6" s="35"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="54"/>
       <c r="J6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1243,15 +1244,15 @@
       </c>
     </row>
     <row r="7" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="42"/>
-      <c r="B7" s="44"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
+      <c r="A7" s="40"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="55"/>
+      <c r="E7" s="56"/>
+      <c r="F7" s="56"/>
+      <c r="G7" s="56"/>
+      <c r="H7" s="56"/>
+      <c r="I7" s="56"/>
       <c r="J7" s="9" t="s">
         <v>34</v>
       </c>
@@ -1266,34 +1267,34 @@
       <c r="A8" s="1"/>
     </row>
     <row r="9" spans="1:21" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="47" t="s">
+      <c r="A9" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="48"/>
-      <c r="C9" s="48"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="47" t="s">
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="48"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="48" t="s">
+      <c r="H9" s="15"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="K9" s="48"/>
-      <c r="L9" s="49"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="16"/>
     </row>
     <row r="10" spans="1:21" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="51" t="s">
+      <c r="B10" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="54"/>
-      <c r="D10" s="52"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="7" t="s">
         <v>7</v>
       </c>
@@ -1312,20 +1313,20 @@
       <c r="J10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K10" s="51" t="s">
+      <c r="K10" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="L10" s="52"/>
+      <c r="L10" s="20"/>
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="55" t="s">
+      <c r="B11" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="55"/>
-      <c r="D11" s="55"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
       <c r="E11" s="12" t="s">
         <v>28</v>
       </c>
@@ -1344,138 +1345,153 @@
       <c r="J11" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="K11" s="53"/>
-      <c r="L11" s="53"/>
+      <c r="K11" s="21"/>
+      <c r="L11" s="21"/>
     </row>
     <row r="12" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
-      <c r="B12" s="56"/>
-      <c r="C12" s="56"/>
-      <c r="D12" s="56"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="18"/>
     </row>
     <row r="13" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="14"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="18"/>
     </row>
     <row r="14" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
-      <c r="B14" s="50"/>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="18"/>
     </row>
     <row r="15" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
       <c r="I15" s="13"/>
       <c r="J15" s="13"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
     </row>
     <row r="16" spans="1:21" s="6" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="18"/>
     </row>
     <row r="17" spans="1:12" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" spans="1:12" ht="114" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="46"/>
+      <c r="K18" s="46"/>
+      <c r="L18" s="46"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="18"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
+      <c r="A19" s="48"/>
+      <c r="B19" s="48"/>
+      <c r="C19" s="48"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="48"/>
+      <c r="H19" s="48"/>
+      <c r="I19" s="48"/>
+      <c r="J19" s="48"/>
+      <c r="K19" s="48"/>
+      <c r="L19" s="48"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
+      <c r="G20" s="49"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="47"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="47"/>
+      <c r="G21" s="47"/>
       <c r="I21" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J21" s="20" t="s">
+      <c r="J21" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="K21" s="21"/>
-      <c r="L21" s="22"/>
+      <c r="K21" s="51"/>
+      <c r="L21" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="D6:I7"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
@@ -1492,21 +1508,6 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="G9:I9"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="D6:I7"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="A18:L18"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="J21:L21"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>